<commit_message>
Updated PA-6 and PA-6,6 calculations to fix bad cell linking
</commit_message>
<xml_diff>
--- a/Article_data/Step 3 - PRODCOM results.xlsx
+++ b/Article_data/Step 3 - PRODCOM results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nicolas\projects\202604-paper-1-supplementary-code\Article_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F85B5D4-79F8-4A42-9EB6-2DF0ECCB430A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{316A3350-7479-474D-BC1B-456BD3C81FAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="570" xr2:uid="{EE4678C9-3BCB-4D41-A2DA-6855614353C7}"/>
+    <workbookView xWindow="-4788" yWindow="-17388" windowWidth="30936" windowHeight="16776" tabRatio="570" activeTab="3" xr2:uid="{EE4678C9-3BCB-4D41-A2DA-6855614353C7}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="4" r:id="rId1"/>
@@ -10225,11 +10225,11 @@
     <xf numFmtId="11" fontId="3" fillId="0" borderId="15" xfId="2" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="4" fillId="0" borderId="14" xfId="4" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="4" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -40806,8 +40806,8 @@
       <c r="D10" s="75" t="s">
         <v>2864</v>
       </c>
-      <c r="F10" s="106">
-        <f>C10/$C$4</f>
+      <c r="F10" s="105">
+        <f t="shared" ref="F10:F16" si="0">C10/$C$4</f>
         <v>9.3484419263456089E-2</v>
       </c>
       <c r="G10" s="50" t="s">
@@ -40830,8 +40830,8 @@
       <c r="E11" s="14" t="s">
         <v>3128</v>
       </c>
-      <c r="F11" s="106">
-        <f>C11/$C$4</f>
+      <c r="F11" s="105">
+        <f t="shared" si="0"/>
         <v>1.69971671388102E-2</v>
       </c>
       <c r="G11" s="50" t="s">
@@ -40854,8 +40854,8 @@
       <c r="E12" s="14" t="s">
         <v>3128</v>
       </c>
-      <c r="F12" s="106">
-        <f>C12/$C$4</f>
+      <c r="F12" s="105">
+        <f t="shared" si="0"/>
         <v>3.6827195467422094E-2</v>
       </c>
       <c r="G12" s="50" t="s">
@@ -40878,8 +40878,8 @@
       <c r="E13" s="14" t="s">
         <v>3128</v>
       </c>
-      <c r="F13" s="106">
-        <f>C13/$C$4</f>
+      <c r="F13" s="105">
+        <f t="shared" si="0"/>
         <v>7.3654390934844188E-2</v>
       </c>
       <c r="G13" s="50" t="s">
@@ -40888,7 +40888,7 @@
       <c r="H13" s="49" t="s">
         <v>3135</v>
       </c>
-      <c r="I13" s="107" t="s">
+      <c r="I13" s="106" t="s">
         <v>3041</v>
       </c>
     </row>
@@ -40905,8 +40905,8 @@
       <c r="E14" s="14" t="s">
         <v>3128</v>
       </c>
-      <c r="F14" s="106">
-        <f>C14/$C$4</f>
+      <c r="F14" s="105">
+        <f t="shared" si="0"/>
         <v>9.6317280453257784E-2</v>
       </c>
       <c r="G14" s="50" t="s">
@@ -40915,7 +40915,7 @@
       <c r="H14" s="49" t="s">
         <v>3136</v>
       </c>
-      <c r="I14" s="107" t="s">
+      <c r="I14" s="106" t="s">
         <v>3041</v>
       </c>
     </row>
@@ -40932,8 +40932,8 @@
       <c r="E15" s="14" t="s">
         <v>3128</v>
       </c>
-      <c r="F15" s="106">
-        <f>C15/$C$4</f>
+      <c r="F15" s="105">
+        <f t="shared" si="0"/>
         <v>0.49291784702549574</v>
       </c>
       <c r="G15" s="50" t="s">
@@ -40959,8 +40959,8 @@
       <c r="E16" s="14" t="s">
         <v>3128</v>
       </c>
-      <c r="F16" s="106">
-        <f>C16/$C$4</f>
+      <c r="F16" s="105">
+        <f t="shared" si="0"/>
         <v>0.18980169971671387</v>
       </c>
       <c r="G16" s="50" t="s">
@@ -40987,7 +40987,7 @@
       <c r="E18" s="14" t="s">
         <v>3128</v>
       </c>
-      <c r="F18" s="106">
+      <c r="F18" s="105">
         <f>SUM(F10:F16)</f>
         <v>1</v>
       </c>
@@ -41115,10 +41115,10 @@
       </c>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.3">
-      <c r="F7" s="105" t="s">
+      <c r="F7" s="107" t="s">
         <v>705</v>
       </c>
-      <c r="G7" s="105"/>
+      <c r="G7" s="107"/>
       <c r="I7" s="47" t="s">
         <v>3072</v>
       </c>

</xml_diff>